<commit_message>
Switched from 500 episodes to 1500 episodes. Retrained and evaluated.
</commit_message>
<xml_diff>
--- a/results/data/Romario_Balanced_replay_experiment_results.xlsx
+++ b/results/data/Romario_Balanced_replay_experiment_results.xlsx
@@ -750,190 +750,190 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>5217.2</v>
+        <v>481.3</v>
       </c>
       <c r="C2" t="n">
-        <v>2506.051906884612</v>
+        <v>70.46282707924796</v>
       </c>
       <c r="D2" t="n">
-        <v>1924.7</v>
+        <v>508.3</v>
       </c>
       <c r="E2" t="n">
-        <v>2209.415354794114</v>
+        <v>4.583666654546335</v>
       </c>
       <c r="F2" t="n">
-        <v>1459.4</v>
+        <v>380.5</v>
       </c>
       <c r="G2" t="n">
-        <v>1326.836553611634</v>
+        <v>104.8200839534104</v>
       </c>
       <c r="H2" t="n">
-        <v>575.6</v>
+        <v>309.3</v>
       </c>
       <c r="I2" t="n">
-        <v>66.38102138412756</v>
+        <v>66.75185390683917</v>
       </c>
       <c r="J2" t="n">
-        <v>573.9</v>
+        <v>306.9</v>
       </c>
       <c r="K2" t="n">
-        <v>45.64088079781107</v>
+        <v>67.11698741749365</v>
       </c>
       <c r="L2" t="n">
-        <v>1101.6</v>
+        <v>287.6</v>
       </c>
       <c r="M2" t="n">
-        <v>1471.721318728515</v>
+        <v>11.85917366429888</v>
       </c>
       <c r="N2" t="n">
-        <v>600.1</v>
+        <v>278.6</v>
       </c>
       <c r="O2" t="n">
-        <v>115.4083619154175</v>
+        <v>37.59308447041823</v>
       </c>
       <c r="P2" t="n">
-        <v>604.2</v>
+        <v>273.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>89.22645347653352</v>
+        <v>46.11333863428238</v>
       </c>
       <c r="R2" t="n">
-        <v>608</v>
+        <v>277.4</v>
       </c>
       <c r="S2" t="n">
-        <v>214.1270650805264</v>
+        <v>38.59844556455609</v>
       </c>
       <c r="T2" t="n">
-        <v>581.5</v>
+        <v>261.4</v>
       </c>
       <c r="U2" t="n">
-        <v>308.6493965650994</v>
+        <v>47.65333146800966</v>
       </c>
       <c r="V2" t="n">
-        <v>577.1</v>
+        <v>267.1</v>
       </c>
       <c r="W2" t="n">
-        <v>234.9682744542335</v>
+        <v>52.82319566251175</v>
       </c>
       <c r="X2" t="n">
-        <v>254.7</v>
+        <v>266.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>89.4506008923361</v>
+        <v>47.70377343565182</v>
       </c>
       <c r="Z2" t="n">
-        <v>239.2</v>
+        <v>259.1</v>
       </c>
       <c r="AA2" t="n">
-        <v>133.6426578604302</v>
+        <v>39.86088308103572</v>
       </c>
       <c r="AB2" t="n">
-        <v>228.4</v>
+        <v>243.9</v>
       </c>
       <c r="AC2" t="n">
-        <v>111.912644504542</v>
+        <v>46.956256239185</v>
       </c>
       <c r="AD2" t="n">
-        <v>192</v>
+        <v>208.3</v>
       </c>
       <c r="AE2" t="n">
-        <v>95.95936640057603</v>
+        <v>55.63640894234638</v>
       </c>
       <c r="AF2" t="n">
-        <v>200.4</v>
+        <v>203.1</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.82701997992939</v>
+        <v>60.61922137408233</v>
       </c>
       <c r="AH2" t="n">
-        <v>201.1</v>
+        <v>232.4</v>
       </c>
       <c r="AI2" t="n">
-        <v>80.80402217711691</v>
+        <v>67.18958252586484</v>
       </c>
       <c r="AJ2" t="n">
-        <v>230.3</v>
+        <v>251.4</v>
       </c>
       <c r="AK2" t="n">
-        <v>128.2295207820727</v>
+        <v>73.6833766870113</v>
       </c>
       <c r="AL2" t="n">
-        <v>198.7</v>
+        <v>178.2</v>
       </c>
       <c r="AM2" t="n">
-        <v>46.02836082243208</v>
+        <v>43.33543584642943</v>
       </c>
       <c r="AN2" t="n">
-        <v>217.5</v>
+        <v>225.6</v>
       </c>
       <c r="AO2" t="n">
-        <v>51.24499975607377</v>
+        <v>74.97092769867531</v>
       </c>
       <c r="AP2" t="n">
-        <v>206.3</v>
+        <v>241</v>
       </c>
       <c r="AQ2" t="n">
-        <v>54.25873201614649</v>
+        <v>72.97122720634484</v>
       </c>
       <c r="AR2" t="n">
-        <v>231.7</v>
+        <v>297.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>100.7432876175877</v>
+        <v>34.40479617727738</v>
       </c>
       <c r="AT2" t="n">
-        <v>228.8</v>
+        <v>297.1</v>
       </c>
       <c r="AU2" t="n">
-        <v>75.92074815226732</v>
+        <v>15.42368308803056</v>
       </c>
       <c r="AV2" t="n">
-        <v>209.1</v>
+        <v>281.4</v>
       </c>
       <c r="AW2" t="n">
-        <v>66.84826100954309</v>
+        <v>7.459222479588606</v>
       </c>
       <c r="AX2" t="n">
-        <v>195.2</v>
+        <v>275.4</v>
       </c>
       <c r="AY2" t="n">
-        <v>96.14967498645017</v>
+        <v>7.364781055808788</v>
       </c>
       <c r="AZ2" t="n">
-        <v>170.1</v>
+        <v>269.9</v>
       </c>
       <c r="BA2" t="n">
-        <v>57.34535726630361</v>
+        <v>3.986226285598949</v>
       </c>
       <c r="BB2" t="n">
-        <v>138.3</v>
+        <v>267.4</v>
       </c>
       <c r="BC2" t="n">
-        <v>58.6771676208046</v>
+        <v>4.63033476111609</v>
       </c>
       <c r="BD2" t="n">
-        <v>146.1</v>
+        <v>262.4</v>
       </c>
       <c r="BE2" t="n">
-        <v>60.35138772223883</v>
+        <v>3.852272056851644</v>
       </c>
       <c r="BF2" t="n">
-        <v>149.6</v>
+        <v>265.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>65.12019655989991</v>
+        <v>4.586937976471886</v>
       </c>
       <c r="BH2" t="n">
-        <v>119.9</v>
+        <v>260.7</v>
       </c>
       <c r="BI2" t="n">
-        <v>47.60766744968713</v>
+        <v>4.026164427839479</v>
       </c>
       <c r="BJ2" t="n">
-        <v>17580.7</v>
+        <v>8418.299999999997</v>
       </c>
       <c r="BK2" t="n">
-        <v>586.0233333333332</v>
+        <v>280.6099999999999</v>
       </c>
     </row>
     <row r="3">
@@ -941,190 +941,190 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>3605</v>
+        <v>481.3</v>
       </c>
       <c r="C3" t="n">
-        <v>3117.70200628604</v>
+        <v>70.12424687652624</v>
       </c>
       <c r="D3" t="n">
-        <v>2225.1</v>
+        <v>508.7</v>
       </c>
       <c r="E3" t="n">
-        <v>2765.633759195168</v>
+        <v>10.85403150907532</v>
       </c>
       <c r="F3" t="n">
-        <v>2348</v>
+        <v>380.8</v>
       </c>
       <c r="G3" t="n">
-        <v>1945.634498049415</v>
+        <v>106.6515822667437</v>
       </c>
       <c r="H3" t="n">
-        <v>555.5</v>
+        <v>314.6</v>
       </c>
       <c r="I3" t="n">
-        <v>52.66165587977651</v>
+        <v>72.22769551910125</v>
       </c>
       <c r="J3" t="n">
-        <v>577.9</v>
+        <v>280.2</v>
       </c>
       <c r="K3" t="n">
-        <v>63.4845650532474</v>
+        <v>37.87822593522564</v>
       </c>
       <c r="L3" t="n">
-        <v>1605.2</v>
+        <v>287</v>
       </c>
       <c r="M3" t="n">
-        <v>3157.165241161761</v>
+        <v>12.01665510863984</v>
       </c>
       <c r="N3" t="n">
-        <v>578.4</v>
+        <v>287.4</v>
       </c>
       <c r="O3" t="n">
-        <v>65.16317978736151</v>
+        <v>10.39422916814903</v>
       </c>
       <c r="P3" t="n">
-        <v>586.8</v>
+        <v>265.8</v>
       </c>
       <c r="Q3" t="n">
-        <v>80.10218473924417</v>
+        <v>46.32450755269828</v>
       </c>
       <c r="R3" t="n">
-        <v>660.2</v>
+        <v>295</v>
       </c>
       <c r="S3" t="n">
-        <v>153.9414174288388</v>
+        <v>14.44991349455075</v>
       </c>
       <c r="T3" t="n">
-        <v>639.2</v>
+        <v>272.7</v>
       </c>
       <c r="U3" t="n">
-        <v>258.2126255627327</v>
+        <v>58.31989368988939</v>
       </c>
       <c r="V3" t="n">
-        <v>456.2</v>
+        <v>264.7</v>
       </c>
       <c r="W3" t="n">
-        <v>148.6807317711344</v>
+        <v>44.46807843835845</v>
       </c>
       <c r="X3" t="n">
-        <v>259.3</v>
+        <v>234.8</v>
       </c>
       <c r="Y3" t="n">
-        <v>143.4845287827228</v>
+        <v>53.73416045682671</v>
       </c>
       <c r="Z3" t="n">
-        <v>216</v>
+        <v>254.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>109.5828453728046</v>
+        <v>57.53963851120373</v>
       </c>
       <c r="AB3" t="n">
-        <v>247.2</v>
+        <v>224</v>
       </c>
       <c r="AC3" t="n">
-        <v>95.28882410860153</v>
+        <v>54.66991860246364</v>
       </c>
       <c r="AD3" t="n">
-        <v>197.8</v>
+        <v>240.4</v>
       </c>
       <c r="AE3" t="n">
-        <v>76.98545317136218</v>
+        <v>60.44700157989642</v>
       </c>
       <c r="AF3" t="n">
-        <v>221.4</v>
+        <v>193.4</v>
       </c>
       <c r="AG3" t="n">
-        <v>23.23015281912713</v>
+        <v>53.35016401099438</v>
       </c>
       <c r="AH3" t="n">
-        <v>210.3</v>
+        <v>191.7</v>
       </c>
       <c r="AI3" t="n">
-        <v>111.0090536848234</v>
+        <v>57.35163467591835</v>
       </c>
       <c r="AJ3" t="n">
-        <v>205.6</v>
+        <v>236.3</v>
       </c>
       <c r="AK3" t="n">
-        <v>75.98447209792273</v>
+        <v>76.66818114446174</v>
       </c>
       <c r="AL3" t="n">
-        <v>192.9</v>
+        <v>223.7</v>
       </c>
       <c r="AM3" t="n">
-        <v>52.27131144327642</v>
+        <v>78.67407450996802</v>
       </c>
       <c r="AN3" t="n">
-        <v>252.1</v>
+        <v>223.5</v>
       </c>
       <c r="AO3" t="n">
-        <v>59.08713904057295</v>
+        <v>71.54334350587762</v>
       </c>
       <c r="AP3" t="n">
-        <v>212.2</v>
+        <v>231.1</v>
       </c>
       <c r="AQ3" t="n">
-        <v>65.29441017422549</v>
+        <v>72.92934937321188</v>
       </c>
       <c r="AR3" t="n">
-        <v>201</v>
+        <v>308.4</v>
       </c>
       <c r="AS3" t="n">
-        <v>88.29042983245692</v>
+        <v>18.51593907961462</v>
       </c>
       <c r="AT3" t="n">
-        <v>217.1</v>
+        <v>292.2</v>
       </c>
       <c r="AU3" t="n">
-        <v>81.90048839903216</v>
+        <v>15.18420231688185</v>
       </c>
       <c r="AV3" t="n">
-        <v>226.3</v>
+        <v>282.2</v>
       </c>
       <c r="AW3" t="n">
-        <v>80.54942582042408</v>
+        <v>6.896375859826668</v>
       </c>
       <c r="AX3" t="n">
-        <v>139.2</v>
+        <v>279.1</v>
       </c>
       <c r="AY3" t="n">
-        <v>51.23826694961492</v>
+        <v>8.371977066380436</v>
       </c>
       <c r="AZ3" t="n">
-        <v>147.2</v>
+        <v>270.9</v>
       </c>
       <c r="BA3" t="n">
-        <v>62.82642756038258</v>
+        <v>5.008991914547277</v>
       </c>
       <c r="BB3" t="n">
-        <v>155.5</v>
+        <v>269.8</v>
       </c>
       <c r="BC3" t="n">
-        <v>91.4147143516841</v>
+        <v>5.325410782277738</v>
       </c>
       <c r="BD3" t="n">
-        <v>145.4</v>
+        <v>264.9</v>
       </c>
       <c r="BE3" t="n">
-        <v>40.25468916784727</v>
+        <v>5.889821729050888</v>
       </c>
       <c r="BF3" t="n">
-        <v>137</v>
+        <v>261.8</v>
       </c>
       <c r="BG3" t="n">
-        <v>95.98437372822724</v>
+        <v>6.177378084592201</v>
       </c>
       <c r="BH3" t="n">
-        <v>159.3</v>
+        <v>263.6</v>
       </c>
       <c r="BI3" t="n">
-        <v>59.43576364445904</v>
+        <v>4.841487374764082</v>
       </c>
       <c r="BJ3" t="n">
-        <v>17580.3</v>
+        <v>8384.299999999999</v>
       </c>
       <c r="BK3" t="n">
-        <v>586.0100000000001</v>
+        <v>279.4766666666666</v>
       </c>
     </row>
     <row r="4">
@@ -1132,190 +1132,190 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>3643</v>
+        <v>501.8</v>
       </c>
       <c r="C4" t="n">
-        <v>2804.807693942671</v>
+        <v>6.384355879804947</v>
       </c>
       <c r="D4" t="n">
-        <v>1673.5</v>
+        <v>484.9</v>
       </c>
       <c r="E4" t="n">
-        <v>1355.064075975745</v>
+        <v>56.30888029431947</v>
       </c>
       <c r="F4" t="n">
-        <v>1636.5</v>
+        <v>425.1</v>
       </c>
       <c r="G4" t="n">
-        <v>1686.074864885898</v>
+        <v>105.1289208543491</v>
       </c>
       <c r="H4" t="n">
-        <v>596.7</v>
+        <v>312.4</v>
       </c>
       <c r="I4" t="n">
-        <v>120.6673526683999</v>
+        <v>63.05267639045942</v>
       </c>
       <c r="J4" t="n">
-        <v>594</v>
+        <v>296.7</v>
       </c>
       <c r="K4" t="n">
-        <v>71.19269625460184</v>
+        <v>77.64927559224233</v>
       </c>
       <c r="L4" t="n">
-        <v>1757</v>
+        <v>289.3</v>
       </c>
       <c r="M4" t="n">
-        <v>3428.045040544246</v>
+        <v>8.591274643497322</v>
       </c>
       <c r="N4" t="n">
-        <v>554.2</v>
+        <v>266</v>
       </c>
       <c r="O4" t="n">
-        <v>45.99304295216832</v>
+        <v>40.13477295313878</v>
       </c>
       <c r="P4" t="n">
-        <v>671.7</v>
+        <v>282.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>128.196762829644</v>
+        <v>39.4361509277972</v>
       </c>
       <c r="R4" t="n">
-        <v>700.1</v>
+        <v>292.7</v>
       </c>
       <c r="S4" t="n">
-        <v>127.0672656509142</v>
+        <v>18.62820442232691</v>
       </c>
       <c r="T4" t="n">
-        <v>940</v>
+        <v>276.8</v>
       </c>
       <c r="U4" t="n">
-        <v>1022.094711854043</v>
+        <v>30.9864486509829</v>
       </c>
       <c r="V4" t="n">
-        <v>437.3</v>
+        <v>231.5</v>
       </c>
       <c r="W4" t="n">
-        <v>356.4609515781498</v>
+        <v>61.59748371484017</v>
       </c>
       <c r="X4" t="n">
-        <v>303.9</v>
+        <v>282.7</v>
       </c>
       <c r="Y4" t="n">
-        <v>159.2434928026888</v>
+        <v>15.65279527752152</v>
       </c>
       <c r="Z4" t="n">
-        <v>239.2</v>
+        <v>242.3</v>
       </c>
       <c r="AA4" t="n">
-        <v>101.6157468112103</v>
+        <v>59.50302513318125</v>
       </c>
       <c r="AB4" t="n">
-        <v>244.8</v>
+        <v>258.4</v>
       </c>
       <c r="AC4" t="n">
-        <v>123.9127112123692</v>
+        <v>59.71130546219869</v>
       </c>
       <c r="AD4" t="n">
-        <v>188.3</v>
+        <v>190.5</v>
       </c>
       <c r="AE4" t="n">
-        <v>60.81455417907789</v>
+        <v>43.71784532659404</v>
       </c>
       <c r="AF4" t="n">
-        <v>205.4</v>
+        <v>229.1</v>
       </c>
       <c r="AG4" t="n">
-        <v>43.70858039332781</v>
+        <v>53.93968854192616</v>
       </c>
       <c r="AH4" t="n">
         <v>216.7</v>
       </c>
       <c r="AI4" t="n">
-        <v>55.36975708814334</v>
+        <v>57.16826042481964</v>
       </c>
       <c r="AJ4" t="n">
-        <v>216.1</v>
+        <v>258.9</v>
       </c>
       <c r="AK4" t="n">
-        <v>47.93422576823371</v>
+        <v>75.60482788817127</v>
       </c>
       <c r="AL4" t="n">
-        <v>212.8</v>
+        <v>161</v>
       </c>
       <c r="AM4" t="n">
-        <v>81.9155662862682</v>
+        <v>7.280109889280518</v>
       </c>
       <c r="AN4" t="n">
-        <v>181.7</v>
+        <v>186.9</v>
       </c>
       <c r="AO4" t="n">
-        <v>50.50356423065603</v>
+        <v>47.15601764356273</v>
       </c>
       <c r="AP4" t="n">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="AQ4" t="n">
-        <v>97.97142440528258</v>
+        <v>70.46843264895283</v>
       </c>
       <c r="AR4" t="n">
-        <v>194.3</v>
+        <v>284.9</v>
       </c>
       <c r="AS4" t="n">
-        <v>73.15333211822957</v>
+        <v>42.62264656259627</v>
       </c>
       <c r="AT4" t="n">
-        <v>214.7</v>
+        <v>291.4</v>
       </c>
       <c r="AU4" t="n">
-        <v>92.79121725680723</v>
+        <v>13.99428454762872</v>
       </c>
       <c r="AV4" t="n">
-        <v>227.7</v>
+        <v>277.4</v>
       </c>
       <c r="AW4" t="n">
-        <v>94.34516415800016</v>
+        <v>7.989993742175271</v>
       </c>
       <c r="AX4" t="n">
-        <v>190.9</v>
+        <v>279.5</v>
       </c>
       <c r="AY4" t="n">
-        <v>131.6635484862838</v>
+        <v>6.726812023536855</v>
       </c>
       <c r="AZ4" t="n">
-        <v>172.4</v>
+        <v>267.2</v>
       </c>
       <c r="BA4" t="n">
-        <v>64.32448989304152</v>
+        <v>5.758472019555188</v>
       </c>
       <c r="BB4" t="n">
-        <v>150.5</v>
+        <v>265.3</v>
       </c>
       <c r="BC4" t="n">
-        <v>59.89866442584509</v>
+        <v>8.258934555982389</v>
       </c>
       <c r="BD4" t="n">
-        <v>164</v>
+        <v>263.9</v>
       </c>
       <c r="BE4" t="n">
-        <v>88.17709453140311</v>
+        <v>5.906775770248943</v>
       </c>
       <c r="BF4" t="n">
-        <v>161.7</v>
+        <v>265.1</v>
       </c>
       <c r="BG4" t="n">
-        <v>71.22085368766651</v>
+        <v>6.533758489567853</v>
       </c>
       <c r="BH4" t="n">
-        <v>174.8</v>
+        <v>261.5</v>
       </c>
       <c r="BI4" t="n">
-        <v>79.47804728351093</v>
+        <v>7.90253124005214</v>
       </c>
       <c r="BJ4" t="n">
-        <v>17116.9</v>
+        <v>8381.199999999997</v>
       </c>
       <c r="BK4" t="n">
-        <v>570.5633333333334</v>
+        <v>279.3733333333332</v>
       </c>
     </row>
     <row r="5">
@@ -1323,190 +1323,190 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>4656.4</v>
+        <v>503.2</v>
       </c>
       <c r="C5" t="n">
-        <v>3363.665120073638</v>
+        <v>4.578209256903839</v>
       </c>
       <c r="D5" t="n">
-        <v>2256.2</v>
+        <v>484.9</v>
       </c>
       <c r="E5" t="n">
-        <v>2277.23625476146</v>
+        <v>61.74050534292703</v>
       </c>
       <c r="F5" t="n">
-        <v>1684.1</v>
+        <v>422.4</v>
       </c>
       <c r="G5" t="n">
-        <v>1680.573678837081</v>
+        <v>106.4999530516329</v>
       </c>
       <c r="H5" t="n">
-        <v>916.4</v>
+        <v>402.5</v>
       </c>
       <c r="I5" t="n">
-        <v>1111.86934484228</v>
+        <v>108.4907830186509</v>
       </c>
       <c r="J5" t="n">
-        <v>573.5</v>
+        <v>274.7</v>
       </c>
       <c r="K5" t="n">
-        <v>90.38500981910661</v>
+        <v>34.44720598248863</v>
       </c>
       <c r="L5" t="n">
-        <v>787.9</v>
+        <v>290.5</v>
       </c>
       <c r="M5" t="n">
-        <v>616.4766743356961</v>
+        <v>7.365459931328117</v>
       </c>
       <c r="N5" t="n">
-        <v>1736.8</v>
+        <v>300.6</v>
       </c>
       <c r="O5" t="n">
-        <v>1648.244144536846</v>
+        <v>20.79038239186572</v>
       </c>
       <c r="P5" t="n">
-        <v>600.3</v>
+        <v>271.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>115.5716660778065</v>
+        <v>52.05391435809607</v>
       </c>
       <c r="R5" t="n">
-        <v>642.1</v>
+        <v>265.6</v>
       </c>
       <c r="S5" t="n">
-        <v>142.9401623057705</v>
+        <v>48.7159111584706</v>
       </c>
       <c r="T5" t="n">
-        <v>656.9</v>
+        <v>271</v>
       </c>
       <c r="U5" t="n">
-        <v>304.2490591604188</v>
+        <v>52.50333322751995</v>
       </c>
       <c r="V5" t="n">
-        <v>416.2</v>
+        <v>264.9</v>
       </c>
       <c r="W5" t="n">
-        <v>208.10036040334</v>
+        <v>49.25941534366806</v>
       </c>
       <c r="X5" t="n">
-        <v>400.6</v>
+        <v>233.8</v>
       </c>
       <c r="Y5" t="n">
-        <v>213.9412068770297</v>
+        <v>67.4207683136287</v>
       </c>
       <c r="Z5" t="n">
-        <v>296.2</v>
+        <v>243.8</v>
       </c>
       <c r="AA5" t="n">
-        <v>192.6555475453536</v>
+        <v>54.59450521801621</v>
       </c>
       <c r="AB5" t="n">
-        <v>219.9</v>
+        <v>267.3</v>
       </c>
       <c r="AC5" t="n">
-        <v>93.86421043187866</v>
+        <v>37.94746368336097</v>
       </c>
       <c r="AD5" t="n">
-        <v>201.4</v>
+        <v>212.7</v>
       </c>
       <c r="AE5" t="n">
-        <v>42.88169772758537</v>
+        <v>54.13326149420521</v>
       </c>
       <c r="AF5" t="n">
-        <v>211.8</v>
+        <v>245.1</v>
       </c>
       <c r="AG5" t="n">
-        <v>57.31631530375972</v>
+        <v>71.08368307846744</v>
       </c>
       <c r="AH5" t="n">
-        <v>195.4</v>
+        <v>234.2</v>
       </c>
       <c r="AI5" t="n">
-        <v>48.7959014672339</v>
+        <v>77.72618606364267</v>
       </c>
       <c r="AJ5" t="n">
-        <v>219.7</v>
+        <v>208.3</v>
       </c>
       <c r="AK5" t="n">
-        <v>36.40068680670737</v>
+        <v>72.04727614559762</v>
       </c>
       <c r="AL5" t="n">
-        <v>205.2</v>
+        <v>221.6</v>
       </c>
       <c r="AM5" t="n">
-        <v>66.51886950332214</v>
+        <v>75.16275673496816</v>
       </c>
       <c r="AN5" t="n">
-        <v>227.1</v>
+        <v>204.5</v>
       </c>
       <c r="AO5" t="n">
-        <v>62.78925067238819</v>
+        <v>52.24413842719583</v>
       </c>
       <c r="AP5" t="n">
-        <v>257.4</v>
+        <v>244.4</v>
       </c>
       <c r="AQ5" t="n">
-        <v>85.34424409413913</v>
+        <v>67.32339860702221</v>
       </c>
       <c r="AR5" t="n">
-        <v>221.8</v>
+        <v>302.5</v>
       </c>
       <c r="AS5" t="n">
-        <v>64.42173546249744</v>
+        <v>13.23820229487373</v>
       </c>
       <c r="AT5" t="n">
-        <v>178.5</v>
+        <v>291.8</v>
       </c>
       <c r="AU5" t="n">
-        <v>85.30914370687353</v>
+        <v>6.64529909033446</v>
       </c>
       <c r="AV5" t="n">
-        <v>217.7</v>
+        <v>281.8</v>
       </c>
       <c r="AW5" t="n">
-        <v>82.49612112093513</v>
+        <v>6.749814812274481</v>
       </c>
       <c r="AX5" t="n">
-        <v>241.3</v>
+        <v>274.3</v>
       </c>
       <c r="AY5" t="n">
-        <v>109.3718885271714</v>
+        <v>5.273518749374084</v>
       </c>
       <c r="AZ5" t="n">
-        <v>215.5</v>
+        <v>270.9</v>
       </c>
       <c r="BA5" t="n">
-        <v>142.4978947212905</v>
+        <v>4.928488612140643</v>
       </c>
       <c r="BB5" t="n">
-        <v>221.3</v>
+        <v>269.3</v>
       </c>
       <c r="BC5" t="n">
-        <v>119.2753536989096</v>
+        <v>6.017474553332153</v>
       </c>
       <c r="BD5" t="n">
-        <v>190.4</v>
+        <v>268.5</v>
       </c>
       <c r="BE5" t="n">
-        <v>93.17961150380484</v>
+        <v>5.661271941887264</v>
       </c>
       <c r="BF5" t="n">
-        <v>184.2</v>
+        <v>264.5</v>
       </c>
       <c r="BG5" t="n">
-        <v>124.6690017606622</v>
+        <v>4.129164564412516</v>
       </c>
       <c r="BH5" t="n">
-        <v>143.1</v>
+        <v>263.4</v>
       </c>
       <c r="BI5" t="n">
-        <v>61.30489376876857</v>
+        <v>8.685620300243384</v>
       </c>
       <c r="BJ5" t="n">
-        <v>19175.3</v>
+        <v>8554.699999999999</v>
       </c>
       <c r="BK5" t="n">
-        <v>639.1766666666666</v>
+        <v>285.1566666666666</v>
       </c>
     </row>
     <row r="6">
@@ -1514,190 +1514,190 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4906.8</v>
+        <v>503.3</v>
       </c>
       <c r="C6" t="n">
-        <v>2158.673889219953</v>
+        <v>7.720751258783046</v>
       </c>
       <c r="D6" t="n">
-        <v>3608.2</v>
+        <v>464.1</v>
       </c>
       <c r="E6" t="n">
-        <v>3670.803857467734</v>
+        <v>80.08052197632081</v>
       </c>
       <c r="F6" t="n">
-        <v>1427.5</v>
+        <v>399.6</v>
       </c>
       <c r="G6" t="n">
-        <v>1371.603094922143</v>
+        <v>110.101044500041</v>
       </c>
       <c r="H6" t="n">
-        <v>568.9</v>
+        <v>376.9</v>
       </c>
       <c r="I6" t="n">
-        <v>75.73697907891496</v>
+        <v>106.267069217138</v>
       </c>
       <c r="J6" t="n">
-        <v>536</v>
+        <v>282.5</v>
       </c>
       <c r="K6" t="n">
-        <v>40.16715075780208</v>
+        <v>37.03849348988157</v>
       </c>
       <c r="L6" t="n">
-        <v>1922.8</v>
+        <v>299.4</v>
       </c>
       <c r="M6" t="n">
-        <v>3316.094443769658</v>
+        <v>14.37497826085313</v>
       </c>
       <c r="N6" t="n">
-        <v>661.6</v>
+        <v>287.6</v>
       </c>
       <c r="O6" t="n">
-        <v>125.6536509616812</v>
+        <v>39.299363862536</v>
       </c>
       <c r="P6" t="n">
-        <v>885.8</v>
+        <v>291.6</v>
       </c>
       <c r="Q6" t="n">
-        <v>724.5821968555397</v>
+        <v>9.254188241007419</v>
       </c>
       <c r="R6" t="n">
-        <v>832.3</v>
+        <v>252.1</v>
       </c>
       <c r="S6" t="n">
-        <v>577.185420813797</v>
+        <v>54.78220513999049</v>
       </c>
       <c r="T6" t="n">
-        <v>663</v>
+        <v>269.9</v>
       </c>
       <c r="U6" t="n">
-        <v>303.1827831523419</v>
+        <v>52.62594417205263</v>
       </c>
       <c r="V6" t="n">
-        <v>564.7</v>
+        <v>278.2</v>
       </c>
       <c r="W6" t="n">
-        <v>204.502836166152</v>
+        <v>37.56008519692148</v>
       </c>
       <c r="X6" t="n">
-        <v>280.6</v>
+        <v>255.5</v>
       </c>
       <c r="Y6" t="n">
-        <v>100.554661751706</v>
+        <v>60.05206074732157</v>
       </c>
       <c r="Z6" t="n">
-        <v>269.9</v>
+        <v>230.6</v>
       </c>
       <c r="AA6" t="n">
-        <v>113.649857017068</v>
+        <v>57.6735641347056</v>
       </c>
       <c r="AB6" t="n">
-        <v>207.9</v>
+        <v>234.6</v>
       </c>
       <c r="AC6" t="n">
-        <v>102.4689709131501</v>
+        <v>52.79810602663698</v>
       </c>
       <c r="AD6" t="n">
-        <v>204.4</v>
+        <v>236</v>
       </c>
       <c r="AE6" t="n">
-        <v>64.78765314471578</v>
+        <v>54.43160846420029</v>
       </c>
       <c r="AF6" t="n">
-        <v>208.6</v>
+        <v>234.2</v>
       </c>
       <c r="AG6" t="n">
-        <v>48.24562156299782</v>
+        <v>71.28646435333989</v>
       </c>
       <c r="AH6" t="n">
-        <v>224.1</v>
+        <v>192.6</v>
       </c>
       <c r="AI6" t="n">
-        <v>62.38661715464303</v>
+        <v>54.86200871276953</v>
       </c>
       <c r="AJ6" t="n">
-        <v>195.7</v>
+        <v>174.1</v>
       </c>
       <c r="AK6" t="n">
-        <v>55.53926538945217</v>
+        <v>39.04983994845561</v>
       </c>
       <c r="AL6" t="n">
-        <v>233.6</v>
+        <v>258.4</v>
       </c>
       <c r="AM6" t="n">
-        <v>27.99714271135538</v>
+        <v>76.10019710881176</v>
       </c>
       <c r="AN6" t="n">
-        <v>225.6</v>
+        <v>245.4</v>
       </c>
       <c r="AO6" t="n">
-        <v>52.44845088274772</v>
+        <v>75.66531570012775</v>
       </c>
       <c r="AP6" t="n">
-        <v>201.2</v>
+        <v>269.7</v>
       </c>
       <c r="AQ6" t="n">
-        <v>67.65175533568956</v>
+        <v>66.93138277370339</v>
       </c>
       <c r="AR6" t="n">
-        <v>186.9</v>
+        <v>313.3</v>
       </c>
       <c r="AS6" t="n">
-        <v>59.63296068450736</v>
+        <v>17.6468127433823</v>
       </c>
       <c r="AT6" t="n">
-        <v>176.1</v>
+        <v>289.4</v>
       </c>
       <c r="AU6" t="n">
-        <v>68.80617704828542</v>
+        <v>17.48256274120016</v>
       </c>
       <c r="AV6" t="n">
-        <v>217.6</v>
+        <v>287</v>
       </c>
       <c r="AW6" t="n">
-        <v>73.37601788050371</v>
+        <v>7.720103626247513</v>
       </c>
       <c r="AX6" t="n">
-        <v>144</v>
+        <v>277.8</v>
       </c>
       <c r="AY6" t="n">
-        <v>80.90488242374498</v>
+        <v>14.09822683886169</v>
       </c>
       <c r="AZ6" t="n">
-        <v>176.7</v>
+        <v>268.9</v>
       </c>
       <c r="BA6" t="n">
-        <v>79.00132910274358</v>
+        <v>4.988987873306568</v>
       </c>
       <c r="BB6" t="n">
-        <v>165.4</v>
+        <v>271</v>
       </c>
       <c r="BC6" t="n">
-        <v>83.47598457041403</v>
+        <v>8.378544026261364</v>
       </c>
       <c r="BD6" t="n">
-        <v>136.3</v>
+        <v>260.4</v>
       </c>
       <c r="BE6" t="n">
-        <v>59.22170210319862</v>
+        <v>4.199999999999999</v>
       </c>
       <c r="BF6" t="n">
-        <v>151</v>
+        <v>263</v>
       </c>
       <c r="BG6" t="n">
-        <v>42.99534858563191</v>
+        <v>6.942621983083913</v>
       </c>
       <c r="BH6" t="n">
-        <v>107.6</v>
+        <v>260.9</v>
       </c>
       <c r="BI6" t="n">
-        <v>25.66787875925862</v>
+        <v>8.745856161634491</v>
       </c>
       <c r="BJ6" t="n">
-        <v>20290.8</v>
+        <v>8527.999999999998</v>
       </c>
       <c r="BK6" t="n">
-        <v>676.3599999999999</v>
+        <v>284.2666666666666</v>
       </c>
     </row>
     <row r="7">
@@ -1705,190 +1705,190 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1970.1</v>
+        <v>503</v>
       </c>
       <c r="C7" t="n">
-        <v>1517.92815706146</v>
+        <v>3.193743884534262</v>
       </c>
       <c r="D7" t="n">
-        <v>2689.7</v>
+        <v>506.1</v>
       </c>
       <c r="E7" t="n">
-        <v>3544.786454781162</v>
+        <v>4.060788100849391</v>
       </c>
       <c r="F7" t="n">
-        <v>3302.4</v>
+        <v>380.7</v>
       </c>
       <c r="G7" t="n">
-        <v>3367.140602944879</v>
+        <v>108.1</v>
       </c>
       <c r="H7" t="n">
-        <v>595.1</v>
+        <v>333.5</v>
       </c>
       <c r="I7" t="n">
-        <v>90.59961368571059</v>
+        <v>89.76998384760911</v>
       </c>
       <c r="J7" t="n">
-        <v>559.9</v>
+        <v>338</v>
       </c>
       <c r="K7" t="n">
-        <v>55.84702319730211</v>
+        <v>89.97888641231341</v>
       </c>
       <c r="L7" t="n">
-        <v>998.3</v>
+        <v>284.1</v>
       </c>
       <c r="M7" t="n">
-        <v>1165.869722567663</v>
+        <v>9.502105029939418</v>
       </c>
       <c r="N7" t="n">
-        <v>617.3</v>
+        <v>297.7</v>
       </c>
       <c r="O7" t="n">
-        <v>78.32375118698032</v>
+        <v>17.97247896090019</v>
       </c>
       <c r="P7" t="n">
-        <v>684.4</v>
+        <v>278.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>202.4802212562995</v>
+        <v>37.92413479566805</v>
       </c>
       <c r="R7" t="n">
-        <v>686.5</v>
+        <v>287.9</v>
       </c>
       <c r="S7" t="n">
-        <v>129.87551732332</v>
+        <v>12.68424219257895</v>
       </c>
       <c r="T7" t="n">
-        <v>970.6</v>
+        <v>276.8</v>
       </c>
       <c r="U7" t="n">
-        <v>1213.342260040422</v>
+        <v>37.23654119275849</v>
       </c>
       <c r="V7" t="n">
-        <v>543.8</v>
+        <v>252.3</v>
       </c>
       <c r="W7" t="n">
-        <v>282.2041105299496</v>
+        <v>52.15179766796155</v>
       </c>
       <c r="X7" t="n">
-        <v>291.6</v>
+        <v>272.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>96.50616560614147</v>
+        <v>31.90235101054466</v>
       </c>
       <c r="Z7" t="n">
-        <v>232.1</v>
+        <v>278.6</v>
       </c>
       <c r="AA7" t="n">
-        <v>91.64545815260024</v>
+        <v>42.14546238920627</v>
       </c>
       <c r="AB7" t="n">
-        <v>189.7</v>
+        <v>259.5</v>
       </c>
       <c r="AC7" t="n">
-        <v>105.6589324193653</v>
+        <v>54.99499977270661</v>
       </c>
       <c r="AD7" t="n">
-        <v>210.1</v>
+        <v>250.8</v>
       </c>
       <c r="AE7" t="n">
-        <v>84.86866323914852</v>
+        <v>63.81347820014201</v>
       </c>
       <c r="AF7" t="n">
-        <v>163.8</v>
+        <v>238.8</v>
       </c>
       <c r="AG7" t="n">
-        <v>47.05911176382317</v>
+        <v>54.77554198727749</v>
       </c>
       <c r="AH7" t="n">
-        <v>215.5</v>
+        <v>233.1</v>
       </c>
       <c r="AI7" t="n">
-        <v>63.19849681756679</v>
+        <v>70.71272869858723</v>
       </c>
       <c r="AJ7" t="n">
-        <v>193.9</v>
+        <v>193.1</v>
       </c>
       <c r="AK7" t="n">
-        <v>42.94752612200149</v>
+        <v>61.85054567261311</v>
       </c>
       <c r="AL7" t="n">
-        <v>221.2</v>
+        <v>189.4</v>
       </c>
       <c r="AM7" t="n">
-        <v>31.09598044763985</v>
+        <v>53.6436389518832</v>
       </c>
       <c r="AN7" t="n">
-        <v>241.6</v>
+        <v>227.2</v>
       </c>
       <c r="AO7" t="n">
-        <v>84.68553595508503</v>
+        <v>81.66737414659541</v>
       </c>
       <c r="AP7" t="n">
-        <v>222.6</v>
+        <v>229.6</v>
       </c>
       <c r="AQ7" t="n">
-        <v>64.6702404510761</v>
+        <v>72.16813701350479</v>
       </c>
       <c r="AR7" t="n">
-        <v>220.8</v>
+        <v>305.2</v>
       </c>
       <c r="AS7" t="n">
-        <v>61.89313370641367</v>
+        <v>9.724196624914574</v>
       </c>
       <c r="AT7" t="n">
-        <v>198.2</v>
+        <v>279.8</v>
       </c>
       <c r="AU7" t="n">
-        <v>71.69490916376142</v>
+        <v>40.13676618762403</v>
       </c>
       <c r="AV7" t="n">
-        <v>272.8</v>
+        <v>283.3</v>
       </c>
       <c r="AW7" t="n">
-        <v>115.8505934382729</v>
+        <v>6.679071791798618</v>
       </c>
       <c r="AX7" t="n">
-        <v>160.8</v>
+        <v>272.9</v>
       </c>
       <c r="AY7" t="n">
-        <v>68.64226103502128</v>
+        <v>5.664803615307418</v>
       </c>
       <c r="AZ7" t="n">
-        <v>151.9</v>
+        <v>270</v>
       </c>
       <c r="BA7" t="n">
-        <v>50.28807015585306</v>
+        <v>7.113367697511496</v>
       </c>
       <c r="BB7" t="n">
-        <v>178.3</v>
+        <v>270.4</v>
       </c>
       <c r="BC7" t="n">
-        <v>85.49742686186526</v>
+        <v>5.003998401278722</v>
       </c>
       <c r="BD7" t="n">
-        <v>128.3</v>
+        <v>265</v>
       </c>
       <c r="BE7" t="n">
-        <v>80.21976065783294</v>
+        <v>5.796550698475776</v>
       </c>
       <c r="BF7" t="n">
-        <v>152.9</v>
+        <v>259.2</v>
       </c>
       <c r="BG7" t="n">
-        <v>56.51097238590042</v>
+        <v>6.20966987850401</v>
       </c>
       <c r="BH7" t="n">
-        <v>141.3</v>
+        <v>283.4</v>
       </c>
       <c r="BI7" t="n">
-        <v>64.42988437053104</v>
+        <v>68.1692012568726</v>
       </c>
       <c r="BJ7" t="n">
-        <v>17405.5</v>
+        <v>8600.6</v>
       </c>
       <c r="BK7" t="n">
-        <v>580.1833333333333</v>
+        <v>286.6866666666667</v>
       </c>
     </row>
     <row r="8">
@@ -1896,190 +1896,190 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>6450.4</v>
+        <v>499.8</v>
       </c>
       <c r="C8" t="n">
-        <v>2784.095371929633</v>
+        <v>12.75774274705365</v>
       </c>
       <c r="D8" t="n">
-        <v>2548.4</v>
+        <v>510.2</v>
       </c>
       <c r="E8" t="n">
-        <v>1432.150215584943</v>
+        <v>4.975942121849891</v>
       </c>
       <c r="F8" t="n">
-        <v>2587.6</v>
+        <v>443.4</v>
       </c>
       <c r="G8" t="n">
-        <v>2021.48075429869</v>
+        <v>97.23291623724963</v>
       </c>
       <c r="H8" t="n">
-        <v>596.7</v>
+        <v>337.1</v>
       </c>
       <c r="I8" t="n">
-        <v>51.67407473772511</v>
+        <v>85.38319506788206</v>
       </c>
       <c r="J8" t="n">
-        <v>992.4</v>
+        <v>290.2</v>
       </c>
       <c r="K8" t="n">
-        <v>1082.409183257422</v>
+        <v>9.075241043630742</v>
       </c>
       <c r="L8" t="n">
-        <v>591.5</v>
+        <v>268.9</v>
       </c>
       <c r="M8" t="n">
-        <v>108.2591797493404</v>
+        <v>46.6378601567439</v>
       </c>
       <c r="N8" t="n">
-        <v>575.6</v>
+        <v>276.4</v>
       </c>
       <c r="O8" t="n">
-        <v>60.8641109357559</v>
+        <v>32.72063569064635</v>
       </c>
       <c r="P8" t="n">
-        <v>630</v>
+        <v>278.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>161.9203507901339</v>
+        <v>38.70465088332408</v>
       </c>
       <c r="R8" t="n">
-        <v>634.2</v>
+        <v>287.7</v>
       </c>
       <c r="S8" t="n">
-        <v>95.33708617322013</v>
+        <v>10.18871925219259</v>
       </c>
       <c r="T8" t="n">
-        <v>825.3</v>
+        <v>268.7</v>
       </c>
       <c r="U8" t="n">
-        <v>420.3653292078213</v>
+        <v>47.63412642213563</v>
       </c>
       <c r="V8" t="n">
-        <v>504.4</v>
+        <v>297.9</v>
       </c>
       <c r="W8" t="n">
-        <v>297.4287141484494</v>
+        <v>12.46956294342348</v>
       </c>
       <c r="X8" t="n">
-        <v>234.8</v>
+        <v>272.1</v>
       </c>
       <c r="Y8" t="n">
-        <v>91.74835148382776</v>
+        <v>37.87994192181398</v>
       </c>
       <c r="Z8" t="n">
-        <v>236.8</v>
+        <v>259.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>101.381260595832</v>
+        <v>55.33037140666959</v>
       </c>
       <c r="AB8" t="n">
-        <v>206.1</v>
+        <v>236.7</v>
       </c>
       <c r="AC8" t="n">
-        <v>84.34743623845362</v>
+        <v>56.92986913738692</v>
       </c>
       <c r="AD8" t="n">
-        <v>237.4</v>
+        <v>256.9</v>
       </c>
       <c r="AE8" t="n">
-        <v>74.11099783432955</v>
+        <v>64.50961168694165</v>
       </c>
       <c r="AF8" t="n">
-        <v>186.1</v>
+        <v>212.1</v>
       </c>
       <c r="AG8" t="n">
-        <v>32.06696119060863</v>
+        <v>53.2680955169227</v>
       </c>
       <c r="AH8" t="n">
-        <v>193</v>
+        <v>231.9</v>
       </c>
       <c r="AI8" t="n">
-        <v>51.69332645516247</v>
+        <v>75.76734124938001</v>
       </c>
       <c r="AJ8" t="n">
-        <v>243.7</v>
+        <v>188.7</v>
       </c>
       <c r="AK8" t="n">
-        <v>83.4494457740733</v>
+        <v>49.26672304913328</v>
       </c>
       <c r="AL8" t="n">
-        <v>188.8</v>
+        <v>222.1</v>
       </c>
       <c r="AM8" t="n">
-        <v>56.13163101140034</v>
+        <v>72.48924058093036</v>
       </c>
       <c r="AN8" t="n">
-        <v>207.6</v>
+        <v>239.2</v>
       </c>
       <c r="AO8" t="n">
-        <v>58.93080688400592</v>
+        <v>75.61719381198962</v>
       </c>
       <c r="AP8" t="n">
-        <v>218</v>
+        <v>298.6</v>
       </c>
       <c r="AQ8" t="n">
-        <v>64.31951492354401</v>
+        <v>43.46308778722469</v>
       </c>
       <c r="AR8" t="n">
-        <v>234.2</v>
+        <v>293.2</v>
       </c>
       <c r="AS8" t="n">
-        <v>61.03081189038861</v>
+        <v>38.82730997635556</v>
       </c>
       <c r="AT8" t="n">
-        <v>164.1</v>
+        <v>279.7</v>
       </c>
       <c r="AU8" t="n">
-        <v>46.84538397750625</v>
+        <v>34.36873579286849</v>
       </c>
       <c r="AV8" t="n">
-        <v>185.7</v>
+        <v>281.7</v>
       </c>
       <c r="AW8" t="n">
-        <v>92.56786699497833</v>
+        <v>10.27667261325377</v>
       </c>
       <c r="AX8" t="n">
-        <v>200.8</v>
+        <v>275.5</v>
       </c>
       <c r="AY8" t="n">
-        <v>103.0890876863308</v>
+        <v>4.883646178829912</v>
       </c>
       <c r="AZ8" t="n">
-        <v>150.6</v>
+        <v>269.7</v>
       </c>
       <c r="BA8" t="n">
-        <v>102.8320961567934</v>
+        <v>7.043436661176133</v>
       </c>
       <c r="BB8" t="n">
-        <v>191</v>
+        <v>267.8</v>
       </c>
       <c r="BC8" t="n">
-        <v>87.30864791073104</v>
+        <v>5.473572873361603</v>
       </c>
       <c r="BD8" t="n">
-        <v>133.5</v>
+        <v>270.1</v>
       </c>
       <c r="BE8" t="n">
-        <v>26.54147697472769</v>
+        <v>4.437341546466758</v>
       </c>
       <c r="BF8" t="n">
-        <v>132.8</v>
+        <v>265.5</v>
       </c>
       <c r="BG8" t="n">
-        <v>32.18011808555089</v>
+        <v>8.546929273136639</v>
       </c>
       <c r="BH8" t="n">
-        <v>127</v>
+        <v>265.9</v>
       </c>
       <c r="BI8" t="n">
-        <v>45.5521678957215</v>
+        <v>6.204030947698439</v>
       </c>
       <c r="BJ8" t="n">
-        <v>20608.5</v>
+        <v>8645.699999999999</v>
       </c>
       <c r="BK8" t="n">
-        <v>686.9499999999999</v>
+        <v>288.1899999999999</v>
       </c>
     </row>
     <row r="9">
@@ -2087,190 +2087,190 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>2929.5</v>
+        <v>478.3</v>
       </c>
       <c r="C9" t="n">
-        <v>2114.90941886408</v>
+        <v>67.62255540868001</v>
       </c>
       <c r="D9" t="n">
-        <v>3167.5</v>
+        <v>506.1</v>
       </c>
       <c r="E9" t="n">
-        <v>2252.895525762347</v>
+        <v>17.13154984232308</v>
       </c>
       <c r="F9" t="n">
-        <v>1273.9</v>
+        <v>429.3</v>
       </c>
       <c r="G9" t="n">
-        <v>1414.246332857187</v>
+        <v>111.5087888912798</v>
       </c>
       <c r="H9" t="n">
-        <v>1044.8</v>
+        <v>292.6</v>
       </c>
       <c r="I9" t="n">
-        <v>1264.353494873961</v>
+        <v>11.12834219459485</v>
       </c>
       <c r="J9" t="n">
-        <v>584.1</v>
+        <v>277.8</v>
       </c>
       <c r="K9" t="n">
-        <v>81.68653499812561</v>
+        <v>36.57813554570544</v>
       </c>
       <c r="L9" t="n">
-        <v>599.6</v>
+        <v>288.5</v>
       </c>
       <c r="M9" t="n">
-        <v>77.05867894014276</v>
+        <v>10.81896483033382</v>
       </c>
       <c r="N9" t="n">
-        <v>1202.1</v>
+        <v>293.8</v>
       </c>
       <c r="O9" t="n">
-        <v>1267.101452133964</v>
+        <v>13.84774349849101</v>
       </c>
       <c r="P9" t="n">
-        <v>626</v>
+        <v>285.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>92.71893010599291</v>
+        <v>7.839005038906405</v>
       </c>
       <c r="R9" t="n">
-        <v>955.5</v>
+        <v>257.2</v>
       </c>
       <c r="S9" t="n">
-        <v>553.8964253360009</v>
+        <v>59.8411229841152</v>
       </c>
       <c r="T9" t="n">
-        <v>625.9</v>
+        <v>276.5</v>
       </c>
       <c r="U9" t="n">
-        <v>253.8989759727282</v>
+        <v>37.79219496139381</v>
       </c>
       <c r="V9" t="n">
-        <v>392.3</v>
+        <v>258.5</v>
       </c>
       <c r="W9" t="n">
-        <v>237.3044668774695</v>
+        <v>57.67885227706945</v>
       </c>
       <c r="X9" t="n">
-        <v>273.4</v>
+        <v>266.3</v>
       </c>
       <c r="Y9" t="n">
-        <v>121.5271163156602</v>
+        <v>47.87076352012782</v>
       </c>
       <c r="Z9" t="n">
-        <v>259.2</v>
+        <v>269.1</v>
       </c>
       <c r="AA9" t="n">
-        <v>127.162730389057</v>
+        <v>37.84296500011594</v>
       </c>
       <c r="AB9" t="n">
-        <v>274</v>
+        <v>261.4</v>
       </c>
       <c r="AC9" t="n">
-        <v>162.1721307746803</v>
+        <v>52.46941966517259</v>
       </c>
       <c r="AD9" t="n">
-        <v>197.8</v>
+        <v>273.2</v>
       </c>
       <c r="AE9" t="n">
-        <v>61.21405067466129</v>
+        <v>34.38837012712292</v>
       </c>
       <c r="AF9" t="n">
-        <v>218.6</v>
+        <v>209.2</v>
       </c>
       <c r="AG9" t="n">
-        <v>74.2040430165365</v>
+        <v>69.49215783093801</v>
       </c>
       <c r="AH9" t="n">
-        <v>182</v>
+        <v>205.7</v>
       </c>
       <c r="AI9" t="n">
-        <v>54.51421832879932</v>
+        <v>65.95612177804271</v>
       </c>
       <c r="AJ9" t="n">
-        <v>206</v>
+        <v>190.6</v>
       </c>
       <c r="AK9" t="n">
-        <v>40.78480109060236</v>
+        <v>49.5745902655786</v>
       </c>
       <c r="AL9" t="n">
-        <v>200.9</v>
+        <v>219.1</v>
       </c>
       <c r="AM9" t="n">
-        <v>42.81693590157987</v>
+        <v>67.7664371204507</v>
       </c>
       <c r="AN9" t="n">
-        <v>228.4</v>
+        <v>228.3</v>
       </c>
       <c r="AO9" t="n">
-        <v>78.43111627409111</v>
+        <v>75.16122670632778</v>
       </c>
       <c r="AP9" t="n">
-        <v>225.3</v>
+        <v>252.9</v>
       </c>
       <c r="AQ9" t="n">
-        <v>59.31618666097813</v>
+        <v>65.51557066835333</v>
       </c>
       <c r="AR9" t="n">
-        <v>223.1</v>
+        <v>286</v>
       </c>
       <c r="AS9" t="n">
-        <v>53.17978939409218</v>
+        <v>29.81945673549403</v>
       </c>
       <c r="AT9" t="n">
-        <v>207.6</v>
+        <v>282.8</v>
       </c>
       <c r="AU9" t="n">
-        <v>84.53780219523098</v>
+        <v>10.06777035892257</v>
       </c>
       <c r="AV9" t="n">
-        <v>236.8</v>
+        <v>279.9</v>
       </c>
       <c r="AW9" t="n">
-        <v>77.30433364307592</v>
+        <v>8.466994744299774</v>
       </c>
       <c r="AX9" t="n">
-        <v>159.1</v>
+        <v>274.5</v>
       </c>
       <c r="AY9" t="n">
-        <v>81.47570189940065</v>
+        <v>6.960603422117942</v>
       </c>
       <c r="AZ9" t="n">
-        <v>225.9</v>
+        <v>269.8</v>
       </c>
       <c r="BA9" t="n">
-        <v>143.3551184994802</v>
+        <v>4.791659420284375</v>
       </c>
       <c r="BB9" t="n">
-        <v>173.1</v>
+        <v>268.3</v>
       </c>
       <c r="BC9" t="n">
-        <v>88.40639117167945</v>
+        <v>8.161494961096281</v>
       </c>
       <c r="BD9" t="n">
-        <v>139.9</v>
+        <v>265.9</v>
       </c>
       <c r="BE9" t="n">
-        <v>90.68566590150837</v>
+        <v>3.806573262134856</v>
       </c>
       <c r="BF9" t="n">
-        <v>159.2</v>
+        <v>262.8</v>
       </c>
       <c r="BG9" t="n">
-        <v>100.4268888296357</v>
+        <v>6.539113089708725</v>
       </c>
       <c r="BH9" t="n">
-        <v>127.8</v>
+        <v>260.6</v>
       </c>
       <c r="BI9" t="n">
-        <v>67.84364377006884</v>
+        <v>9.645724441429994</v>
       </c>
       <c r="BJ9" t="n">
-        <v>17319.3</v>
+        <v>8470.5</v>
       </c>
       <c r="BK9" t="n">
-        <v>577.3099999999999</v>
+        <v>282.35</v>
       </c>
     </row>
     <row r="10">
@@ -2278,190 +2278,190 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>5992</v>
+        <v>478.4</v>
       </c>
       <c r="C10" t="n">
-        <v>2982.326541477308</v>
+        <v>60.29792699587608</v>
       </c>
       <c r="D10" t="n">
-        <v>2007</v>
+        <v>503.4</v>
       </c>
       <c r="E10" t="n">
-        <v>1436.554071380538</v>
+        <v>7.735631842325486</v>
       </c>
       <c r="F10" t="n">
-        <v>890.3</v>
+        <v>469.3</v>
       </c>
       <c r="G10" t="n">
-        <v>998.9079086682615</v>
+        <v>85.72403396947674</v>
       </c>
       <c r="H10" t="n">
-        <v>985.4</v>
+        <v>287.3</v>
       </c>
       <c r="I10" t="n">
-        <v>1221.177480958439</v>
+        <v>10.22790301088155</v>
       </c>
       <c r="J10" t="n">
-        <v>583.5</v>
+        <v>286.7</v>
       </c>
       <c r="K10" t="n">
-        <v>61.97781861279082</v>
+        <v>6.356886030125128</v>
       </c>
       <c r="L10" t="n">
-        <v>553.6</v>
+        <v>279.7</v>
       </c>
       <c r="M10" t="n">
-        <v>54.02443891425435</v>
+        <v>35.38940519421032</v>
       </c>
       <c r="N10" t="n">
-        <v>601.1</v>
+        <v>288.3</v>
       </c>
       <c r="O10" t="n">
-        <v>107.8382585170959</v>
+        <v>38.10524898225965</v>
       </c>
       <c r="P10" t="n">
-        <v>568</v>
+        <v>288.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>77.26059797852977</v>
+        <v>12.71259218255663</v>
       </c>
       <c r="R10" t="n">
-        <v>621.9</v>
+        <v>279.5</v>
       </c>
       <c r="S10" t="n">
-        <v>121.5552960590364</v>
+        <v>41.39142423256295</v>
       </c>
       <c r="T10" t="n">
-        <v>587</v>
+        <v>257.3</v>
       </c>
       <c r="U10" t="n">
-        <v>233.5945204836792</v>
+        <v>44.08639245844459</v>
       </c>
       <c r="V10" t="n">
-        <v>417.3</v>
+        <v>265.1</v>
       </c>
       <c r="W10" t="n">
-        <v>222.6724275701866</v>
+        <v>51.0929545045107</v>
       </c>
       <c r="X10" t="n">
-        <v>383</v>
+        <v>251.2</v>
       </c>
       <c r="Y10" t="n">
-        <v>242.6722068964635</v>
+        <v>51.46610535099776</v>
       </c>
       <c r="Z10" t="n">
-        <v>178</v>
+        <v>255.9</v>
       </c>
       <c r="AA10" t="n">
-        <v>89.74185199782764</v>
+        <v>56.79163670823372</v>
       </c>
       <c r="AB10" t="n">
-        <v>263.1</v>
+        <v>250.5</v>
       </c>
       <c r="AC10" t="n">
-        <v>120.6991714967423</v>
+        <v>66.04278915975611</v>
       </c>
       <c r="AD10" t="n">
-        <v>230.6</v>
+        <v>242.6</v>
       </c>
       <c r="AE10" t="n">
-        <v>91.79673196797367</v>
+        <v>61.80485417829249</v>
       </c>
       <c r="AF10" t="n">
-        <v>203.6</v>
+        <v>256</v>
       </c>
       <c r="AG10" t="n">
-        <v>52.39122063857646</v>
+        <v>63.14269553954757</v>
       </c>
       <c r="AH10" t="n">
-        <v>242.9</v>
+        <v>172.4</v>
       </c>
       <c r="AI10" t="n">
-        <v>56.35503526748963</v>
+        <v>33.74077651744251</v>
       </c>
       <c r="AJ10" t="n">
-        <v>220.8</v>
+        <v>212</v>
       </c>
       <c r="AK10" t="n">
-        <v>38.43123729467996</v>
+        <v>60.94751840723296</v>
       </c>
       <c r="AL10" t="n">
-        <v>203.1</v>
+        <v>206.2</v>
       </c>
       <c r="AM10" t="n">
-        <v>49.77640003053656</v>
+        <v>64.54269904489585</v>
       </c>
       <c r="AN10" t="n">
-        <v>231</v>
+        <v>234.4</v>
       </c>
       <c r="AO10" t="n">
-        <v>53.10932121577153</v>
+        <v>80.07771225503386</v>
       </c>
       <c r="AP10" t="n">
-        <v>219.6</v>
+        <v>260.9</v>
       </c>
       <c r="AQ10" t="n">
-        <v>63.96749174385377</v>
+        <v>73.07728785334058</v>
       </c>
       <c r="AR10" t="n">
-        <v>172.8</v>
+        <v>302.4</v>
       </c>
       <c r="AS10" t="n">
-        <v>66.55043200460837</v>
+        <v>19.07983228437818</v>
       </c>
       <c r="AT10" t="n">
-        <v>239.5</v>
+        <v>297.6</v>
       </c>
       <c r="AU10" t="n">
-        <v>65.97006897070823</v>
+        <v>20.11069367277022</v>
       </c>
       <c r="AV10" t="n">
-        <v>195.1</v>
+        <v>279.5</v>
       </c>
       <c r="AW10" t="n">
-        <v>109.9831350707916</v>
+        <v>4.080441152620633</v>
       </c>
       <c r="AX10" t="n">
-        <v>199.6</v>
+        <v>274.5</v>
       </c>
       <c r="AY10" t="n">
-        <v>94.43431579674838</v>
+        <v>3.5</v>
       </c>
       <c r="AZ10" t="n">
-        <v>171.3</v>
+        <v>269.9</v>
       </c>
       <c r="BA10" t="n">
-        <v>82.33717265002484</v>
+        <v>4.482186966202994</v>
       </c>
       <c r="BB10" t="n">
-        <v>164.8</v>
+        <v>267.1</v>
       </c>
       <c r="BC10" t="n">
-        <v>86.14267235232489</v>
+        <v>6.268173577685928</v>
       </c>
       <c r="BD10" t="n">
-        <v>214.6</v>
+        <v>262.1</v>
       </c>
       <c r="BE10" t="n">
-        <v>104.7389134944601</v>
+        <v>4.504442251822083</v>
       </c>
       <c r="BF10" t="n">
-        <v>188.1</v>
+        <v>265.2</v>
       </c>
       <c r="BG10" t="n">
-        <v>99.46904040956663</v>
+        <v>7.756287771866126</v>
       </c>
       <c r="BH10" t="n">
-        <v>148</v>
+        <v>262.7</v>
       </c>
       <c r="BI10" t="n">
-        <v>70.70502103811299</v>
+        <v>8.49764673306675</v>
       </c>
       <c r="BJ10" t="n">
-        <v>17876.59999999999</v>
+        <v>8506.4</v>
       </c>
       <c r="BK10" t="n">
-        <v>595.8866666666664</v>
+        <v>283.5466666666667</v>
       </c>
     </row>
     <row r="11">
@@ -2469,190 +2469,190 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>3670</v>
+        <v>502</v>
       </c>
       <c r="C11" t="n">
-        <v>3008.460370355574</v>
+        <v>2.23606797749979</v>
       </c>
       <c r="D11" t="n">
-        <v>3447</v>
+        <v>506.5</v>
       </c>
       <c r="E11" t="n">
-        <v>3342.131984228031</v>
+        <v>4.695742752749559</v>
       </c>
       <c r="F11" t="n">
-        <v>1823.8</v>
+        <v>447.9</v>
       </c>
       <c r="G11" t="n">
-        <v>2615.734764841421</v>
+        <v>95.50963302201511</v>
       </c>
       <c r="H11" t="n">
-        <v>774.3</v>
+        <v>287.3</v>
       </c>
       <c r="I11" t="n">
-        <v>581.4408052415998</v>
+        <v>4.817675788178362</v>
       </c>
       <c r="J11" t="n">
-        <v>582.4</v>
+        <v>257.5</v>
       </c>
       <c r="K11" t="n">
-        <v>70.35652066439899</v>
+        <v>54.32540842000178</v>
       </c>
       <c r="L11" t="n">
-        <v>669.2</v>
+        <v>268.2</v>
       </c>
       <c r="M11" t="n">
-        <v>171.3842466506184</v>
+        <v>50.78149269172776</v>
       </c>
       <c r="N11" t="n">
-        <v>723.9</v>
+        <v>279.9</v>
       </c>
       <c r="O11" t="n">
-        <v>505.5085459218271</v>
+        <v>38.46153923076923</v>
       </c>
       <c r="P11" t="n">
-        <v>660.3</v>
+        <v>276.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>139.2853545782901</v>
+        <v>39.07991811659794</v>
       </c>
       <c r="R11" t="n">
-        <v>1921.6</v>
+        <v>284.3</v>
       </c>
       <c r="S11" t="n">
-        <v>1827.477124343832</v>
+        <v>39.56526254178026</v>
       </c>
       <c r="T11" t="n">
-        <v>818.9</v>
+        <v>283.5</v>
       </c>
       <c r="U11" t="n">
-        <v>498.003102399975</v>
+        <v>39.38337212580964</v>
       </c>
       <c r="V11" t="n">
-        <v>421.6</v>
+        <v>270.6</v>
       </c>
       <c r="W11" t="n">
-        <v>165.4117287256257</v>
+        <v>51.74591771338103</v>
       </c>
       <c r="X11" t="n">
-        <v>261.3</v>
+        <v>272.3</v>
       </c>
       <c r="Y11" t="n">
-        <v>196.2503757958186</v>
+        <v>30.74752022521491</v>
       </c>
       <c r="Z11" t="n">
-        <v>173.2</v>
+        <v>261.5</v>
       </c>
       <c r="AA11" t="n">
-        <v>67.59704135537294</v>
+        <v>48.1814279572534</v>
       </c>
       <c r="AB11" t="n">
-        <v>286.3</v>
+        <v>231.2</v>
       </c>
       <c r="AC11" t="n">
-        <v>116.3340448879863</v>
+        <v>65.30053598554915</v>
       </c>
       <c r="AD11" t="n">
-        <v>168.6</v>
+        <v>203.9</v>
       </c>
       <c r="AE11" t="n">
-        <v>56.25513309912261</v>
+        <v>58.6642139638809</v>
       </c>
       <c r="AF11" t="n">
-        <v>217.8</v>
+        <v>208.9</v>
       </c>
       <c r="AG11" t="n">
-        <v>57.42960908799571</v>
+        <v>63.88184405603833</v>
       </c>
       <c r="AH11" t="n">
-        <v>173.3</v>
+        <v>201</v>
       </c>
       <c r="AI11" t="n">
-        <v>54.28268600576062</v>
+        <v>58.704343961925</v>
       </c>
       <c r="AJ11" t="n">
-        <v>197.4</v>
+        <v>195.1</v>
       </c>
       <c r="AK11" t="n">
-        <v>47.8919617472494</v>
+        <v>61.01876760472961</v>
       </c>
       <c r="AL11" t="n">
-        <v>211.9</v>
+        <v>198.8</v>
       </c>
       <c r="AM11" t="n">
-        <v>51.3934820770105</v>
+        <v>68.51539972882009</v>
       </c>
       <c r="AN11" t="n">
-        <v>222.6</v>
+        <v>230.8</v>
       </c>
       <c r="AO11" t="n">
-        <v>39.52012145730324</v>
+        <v>71.17134254740458</v>
       </c>
       <c r="AP11" t="n">
-        <v>268.4</v>
+        <v>284.9</v>
       </c>
       <c r="AQ11" t="n">
-        <v>51.21367005009503</v>
+        <v>57.09719782966587</v>
       </c>
       <c r="AR11" t="n">
-        <v>214.6</v>
+        <v>306.1</v>
       </c>
       <c r="AS11" t="n">
-        <v>74.18517372089924</v>
+        <v>13.66345490716019</v>
       </c>
       <c r="AT11" t="n">
-        <v>193.8</v>
+        <v>288</v>
       </c>
       <c r="AU11" t="n">
-        <v>108.9383311786994</v>
+        <v>11.08151614175605</v>
       </c>
       <c r="AV11" t="n">
-        <v>238.6</v>
+        <v>280.8</v>
       </c>
       <c r="AW11" t="n">
-        <v>81.80611224107891</v>
+        <v>7.884161337770808</v>
       </c>
       <c r="AX11" t="n">
-        <v>157.7</v>
+        <v>274.9</v>
       </c>
       <c r="AY11" t="n">
-        <v>75.98953875369951</v>
+        <v>6.564297372910523</v>
       </c>
       <c r="AZ11" t="n">
-        <v>141.6</v>
+        <v>268.5</v>
       </c>
       <c r="BA11" t="n">
-        <v>104.0463358316861</v>
+        <v>1.20415945787923</v>
       </c>
       <c r="BB11" t="n">
-        <v>139.5</v>
+        <v>267.7</v>
       </c>
       <c r="BC11" t="n">
-        <v>53.68286505021877</v>
+        <v>5.254521862167861</v>
       </c>
       <c r="BD11" t="n">
-        <v>140.4</v>
+        <v>263.6</v>
       </c>
       <c r="BE11" t="n">
-        <v>78.77334574588031</v>
+        <v>5.462600113499064</v>
       </c>
       <c r="BF11" t="n">
-        <v>125.2</v>
+        <v>270.1</v>
       </c>
       <c r="BG11" t="n">
-        <v>97.98959128397262</v>
+        <v>5.734980383575867</v>
       </c>
       <c r="BH11" t="n">
-        <v>111.3</v>
+        <v>260.3</v>
       </c>
       <c r="BI11" t="n">
-        <v>44.39155325059037</v>
+        <v>8.34326075344646</v>
       </c>
       <c r="BJ11" t="n">
-        <v>19156.5</v>
+        <v>8432.700000000001</v>
       </c>
       <c r="BK11" t="n">
-        <v>638.5499999999998</v>
+        <v>281.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>